<commit_message>
Sendus Msg Test Added
</commit_message>
<xml_diff>
--- a/tests/testdata/TestData.xlsx
+++ b/tests/testdata/TestData.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{209DAC2C-1FC9-40FD-8300-474F7ED2D79C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D03CC35D-5375-48C0-A3F6-9A80830C0AD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{85C43414-944F-449E-A662-147F6DC72B31}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{85C43414-944F-449E-A662-147F6DC72B31}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="41">
   <si>
     <t>Name</t>
   </si>
@@ -123,6 +124,45 @@
   </si>
   <si>
     <t>Tuesday</t>
+  </si>
+  <si>
+    <t>Full Name</t>
+  </si>
+  <si>
+    <t>Email Address</t>
+  </si>
+  <si>
+    <t>Phone Number</t>
+  </si>
+  <si>
+    <t>Interested Course</t>
+  </si>
+  <si>
+    <t>Your Message</t>
+  </si>
+  <si>
+    <t>Dinesh</t>
+  </si>
+  <si>
+    <t>Dinesh123@gmail.com</t>
+  </si>
+  <si>
+    <t>Playwright with Python</t>
+  </si>
+  <si>
+    <t>I want to join Course</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>Test1234@gmail.com</t>
+  </si>
+  <si>
+    <t>Yogesh</t>
+  </si>
+  <si>
+    <t>Yogesh1@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -167,10 +207,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -689,4 +732,93 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AFDBE5F-6F67-456F-9F96-2165FAA79B1D}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="13.54296875" customWidth="1"/>
+    <col min="3" max="3" width="12.7265625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="21.08984375" customWidth="1"/>
+    <col min="5" max="5" width="17.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="3">
+        <v>8373747655</v>
+      </c>
+      <c r="D2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="3">
+        <v>837373741</v>
+      </c>
+      <c r="D3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="3">
+        <v>999933444</v>
+      </c>
+      <c r="D4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{A91539B5-04C2-4F19-A2E9-B417F299294A}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{96052FC0-3E13-4A2E-B66E-920569EB71B1}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{346E2F98-B908-46E7-9249-304A8504359E}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>